<commit_message>
Actualización del archivo de Parametros
</commit_message>
<xml_diff>
--- a/Parámetros.xlsx
+++ b/Parámetros.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pancanal-my.sharepoint.com/personal/joluflores_pancanal_com/Documents/Documents/Visual Studio Code/apinputvalidator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_5F141882AFA6075A60101E794757A9A6713C159B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21256558-4C6C-4F0A-9837-4AB132A60601}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_5F141882AFA6075A60101E794757A9A6713C159B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{121EDF58-2F46-4561-94A6-0D242808C512}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2244" yWindow="636" windowWidth="9792" windowHeight="11796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
   <si>
     <t>VENDOR_TYPE_LOOKUP_CODE</t>
   </si>
@@ -281,7 +281,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -624,8 +624,8 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
+      <c r="C2">
+        <v>10020</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -644,8 +644,8 @@
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
+      <c r="C3">
+        <v>10087</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -664,8 +664,8 @@
       <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
+      <c r="C4">
+        <v>10087</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -684,8 +684,8 @@
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
-        <v>6</v>
+      <c r="C5">
+        <v>10087</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -704,8 +704,8 @@
       <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
+      <c r="C6">
+        <v>10087</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -724,8 +724,8 @@
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
-        <v>6</v>
+      <c r="C7">
+        <v>10087</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>

</xml_diff>